<commit_message>
Projection multi-villas : commission agence activable et occupation par villa
Cout foncier : les prix saisis sont desormais des prix vendeur et la
commission agence apparait sur sa propre ligne, activable par OUI / NON avec
un taux modifiable (25% par defaut). Les frais de notaire portent sur le prix
commission comprise.

Le forfait plancher des honoraires du notaire passe de 10 a 20 millions IDR,
dans la projection comme dans les deux recapitulatifs d'appel de fonds.

Tableau 2 reorganise en une ligne par villa (designation, construction,
ameublement) et tableau 3 en une grille ou chaque villa a son propre taux
d'occupation et son propre prix de nuitee. Les designations saisies une seule
fois sont reprises automatiquement, et le nombre de villas du scenario est
compte automatiquement.

Co-Authored-By: Claude Opus 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_014vwehdk7pAYrgh8aPNjCvp
</commit_message>
<xml_diff>
--- a/transactions/Recap_transaction_fonciere_FREEHOLD_appel_de_fonds.xlsx
+++ b/transactions/Recap_transaction_fonciere_FREEHOLD_appel_de_fonds.xlsx
@@ -178,12 +178,12 @@
     </comment>
     <comment ref="B15" authorId="0" shapeId="0">
       <text>
-        <t>Forfait plancher : si le pourcentage donne moins de 10 000 000 IDR, ce forfait s'applique a la place du pourcentage.</t>
+        <t>Forfait plancher : si le pourcentage donne moins de 20 000 000 IDR, ce forfait s'applique a la place du pourcentage.</t>
       </text>
     </comment>
     <comment ref="D27" authorId="0" shapeId="0">
       <text>
-        <t>MAX entre le pourcentage d'honoraires et le forfait minimum : si le pourcentage donne moins de 10 000 000 IDR, c'est le forfait qui s'applique.
+        <t>MAX entre le pourcentage d'honoraires et le forfait minimum : si le pourcentage donne moins de 20 000 000 IDR, c'est le forfait qui s'applique.
 La colonne des taux affiche le taux reellement supporte.</t>
       </text>
     </comment>
@@ -606,7 +606,7 @@
         </is>
       </c>
       <c r="B15" s="4" t="n">
-        <v>10000000</v>
+        <v>20000000</v>
       </c>
     </row>
     <row r="16">
@@ -753,7 +753,7 @@
     <row r="27">
       <c r="A27" s="2" t="inlineStr">
         <is>
-          <t>Honoraires du notaire (1% du prix client, minimum 10 000 000 IDR)</t>
+          <t>Honoraires du notaire (1% du prix client, minimum 20 000 000 IDR)</t>
         </is>
       </c>
       <c r="C27" s="5">
@@ -919,7 +919,7 @@
     <row r="45">
       <c r="A45" s="2" t="inlineStr">
         <is>
-          <t>Honoraires du notaire : le pourcentage s'applique sauf s'il donne moins que le forfait minimum de 10 000 000 IDR (B15), auquel cas le forfait est retenu (formule MAX en D27).</t>
+          <t>Honoraires du notaire : le pourcentage s'applique sauf s'il donne moins que le forfait minimum de 20 000 000 IDR (B15), auquel cas le forfait est retenu (formule MAX en D27).</t>
         </is>
       </c>
     </row>

</xml_diff>